<commit_message>
add bai tap ngay 16/06/2026
</commit_message>
<xml_diff>
--- a/AI_AuditLog_Example.xlsx
+++ b/AI_AuditLog_Example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kì 5\SWR302-audit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{503C615B-FBFD-49DF-9E13-597E004946DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF524F8-0216-46E7-BCBE-80573A49D79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="168">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -195,75 +195,18 @@
     <t>DECISION</t>
   </si>
   <si>
-    <t>Cần chia nhỏ requirement</t>
-  </si>
-  <si>
-    <t>Break down student management into modules</t>
-  </si>
-  <si>
-    <t>AI suggested 10 modules: User, Student, Course, Grade, Attendance, Report, Export, Import, Settings, Dashboard</t>
-  </si>
-  <si>
-    <t>Critical Thinking: 10 modules quá nhiều cho project 300 LOC.
-Contextualization: Project scope nhỏ, chỉ cần core functions.
-Creative Synthesis: Tôi gộp thành 5 modules: Student, Grade, File I/O, Validation, UI.
-Decision: Chọn 5 modules vì đủ để implement requirements mà không phức tạp.</t>
-  </si>
-  <si>
-    <t>Screenshot comparison 10 vs 5</t>
-  </si>
-  <si>
     <t>002</t>
   </si>
   <si>
     <t>PROBLEM-SOLVING</t>
   </si>
   <si>
-    <t>Search by name quá chậm với 10K records</t>
-  </si>
-  <si>
-    <t>How to optimize search for player name in 10,000 records?</t>
-  </si>
-  <si>
-    <t>AI suggested Binary Search with O(log n) complexity</t>
-  </si>
-  <si>
-    <t>Critical Thinking: Binary Search cần sort trước → O(n log n). Với partial match không phù hợp.
-Contextualization: Requirements yêu cầu partial name search.
-Creative Synthesis: Test 3 approaches: Binary Search, Linear Search, HashMap. HashMap fastest (2ms).
-Decision: Chọn HashMap trade-off memory cho speed.</t>
-  </si>
-  <si>
-    <t>Code snippet + timing comparison</t>
-  </si>
-  <si>
     <t>003</t>
   </si>
   <si>
     <t>VERIFICATION</t>
   </si>
   <si>
-    <t>Literature Review</t>
-  </si>
-  <si>
-    <t>Cần verify paper AI cite</t>
-  </si>
-  <si>
-    <t>Is the paper 'Smith et al. 2023 on IoT anomaly detection' a real publication?</t>
-  </si>
-  <si>
-    <t>AI confirmed it exists and provided summary</t>
-  </si>
-  <si>
-    <t>Critical Thinking: HALLUCINATION DETECTED! Search Google Scholar → paper NOT FOUND.
-Contextualization: AI fabricated paper to answer my question.
-Creative Synthesis: Found real paper 'Jones et al. 2022' with similar topic.
-Decision: Replace with verified paper from Google Scholar.</t>
-  </si>
-  <si>
-    <t>Google Scholar screenshot</t>
-  </si>
-  <si>
     <t>HALLUCINATION DETECTION LOG (BẮT BUỘC)</t>
   </si>
   <si>
@@ -291,18 +234,6 @@
     <t>Fabrication</t>
   </si>
   <si>
-    <t>Paper 'Smith et al. 2023' exists</t>
-  </si>
-  <si>
-    <t>Paper NOT FOUND on Google Scholar</t>
-  </si>
-  <si>
-    <t>Searched Google Scholar, ResearchGate</t>
-  </si>
-  <si>
-    <t>Used real paper 'Jones et al. 2022'</t>
-  </si>
-  <si>
     <t>HALLUCINATION TYPES REFERENCE:</t>
   </si>
   <si>
@@ -384,9 +315,6 @@
     <t>Prompt này ảnh hưởng đến quyết định quan trọng trong project?</t>
   </si>
   <si>
-    <t>☐</t>
-  </si>
-  <si>
     <t>2</t>
   </si>
   <si>
@@ -463,6 +391,153 @@
   </si>
   <si>
     <t>SWR302</t>
+  </si>
+  <si>
+    <t>Requirement Prioritization</t>
+  </si>
+  <si>
+    <t>Cần phân loại MoSCoW cho hệ thống đặt lịch khám bệnh</t>
+  </si>
+  <si>
+    <t>Classify the 10 requirements using MoSCoW for a clinic booking system MVP</t>
+  </si>
+  <si>
+    <t>AI suggested Must, Should, Could and Won't priorities for all requirements</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI xếp nhiều chức năng vào Must Have. Contextualization: Dự án chỉ có 3 developer và 8 tuần nên cần tập trung MVP. Creative Synthesis: So sánh mức độ ảnh hưởng của từng requirement đến chức năng đặt lịch khám. Decision: Chọn R01, R02, R07, R08 là Must Have và điều chỉnh các requirement còn lại theo phạm vi dự án.</t>
+  </si>
+  <si>
+    <t>Screenshot of MoSCoW classification</t>
+  </si>
+  <si>
+    <t>Requirement Validation</t>
+  </si>
+  <si>
+    <t>Cần tạo câu hỏi Games People Play cho các requirement Should Have</t>
+  </si>
+  <si>
+    <t>Generate Games People Play questions for SMS reminder and appointment history requirements</t>
+  </si>
+  <si>
+    <t>AI suggested questions about business value, impact and alternatives</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Không sử dụng nguyên văn tất cả câu hỏi của AI. Contextualization: Điều chỉnh câu hỏi phù hợp với ngữ cảnh phòng khám tư nhân. Creative Synthesis: Tập trung vào mức độ ảnh hưởng nếu requirement bị loại bỏ. Decision: Chọn 3 câu hỏi cho R03 và 3 câu hỏi cho R04.</t>
+  </si>
+  <si>
+    <t>Screenshot of section 1b</t>
+  </si>
+  <si>
+    <t>Validation vs Verification Analysis</t>
+  </si>
+  <si>
+    <t>Cần phân biệt TH1–TH5 thuộc Verification hay Validation</t>
+  </si>
+  <si>
+    <t>Classify five scenarios as Verification, Validation or both</t>
+  </si>
+  <si>
+    <t>AI classified the scenarios and explained each answer</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Đối chiếu định nghĩa trong Chapter 17 trước khi chấp nhận kết quả. Contextualization: So sánh từng tình huống với khái niệm "Build the product right" và "Build the right product". Creative Synthesis: Tóm tắt lại bằng ngôn ngữ dễ hiểu. Decision: Giữ nguyên phân loại của AI vì phù hợp với lý thuyết môn học.</t>
+  </si>
+  <si>
+    <t>Screenshot of Exercise 2 answers</t>
+  </si>
+  <si>
+    <t>Acceptance Criteria</t>
+  </si>
+  <si>
+    <t>Cần viết Acceptance Criteria theo định dạng Given-When-Then</t>
+  </si>
+  <si>
+    <t>Create 4 testable acceptance criteria for online clinic appointment booking</t>
+  </si>
+  <si>
+    <t>AI generated 4 acceptance criteria including success and failure scenarios</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Loại bỏ các AC quá chung chung và chỉ giữ các AC có thể kiểm thử được. Contextualization: Bổ sung trường hợp khung giờ đã được đặt trước. Creative Synthesis: Kết hợp luồng thành công và luồng lỗi để tăng độ bao phủ kiểm thử. Decision: Chọn 4 AC cuối cùng để sử dụng trong bài tập.</t>
+  </si>
+  <si>
+    <t>Screenshot of Exercise 3a</t>
+  </si>
+  <si>
+    <t>Test Case Design</t>
+  </si>
+  <si>
+    <t>Cần chọn AC phù hợp để thiết kế test case</t>
+  </si>
+  <si>
+    <t>Which acceptance criteria should be used for a detailed test case?</t>
+  </si>
+  <si>
+    <t>AI suggested using the appointment conflict scenario</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Đây là trường hợp dễ bị bỏ sót và có rủi ro cao. Contextualization: Nhiều bệnh nhân có thể chọn cùng một khung giờ. Creative Synthesis: Xây dựng test case với dữ liệu cụ thể và expected result rõ ràng. Decision: Chọn AC về khung giờ đã được đặt trước để thiết kế test case.</t>
+  </si>
+  <si>
+    <t>Screenshot of Exercise 3c</t>
+  </si>
+  <si>
+    <t>Chapter 16 &amp; 17 - MoSCoW Prioritization, Validation &amp; Verification, Acceptance Criteria</t>
+  </si>
+  <si>
+    <t>Misclassification Risk</t>
+  </si>
+  <si>
+    <t>AI initially suggested focusing only on Verification because all tests passed.</t>
+  </si>
+  <si>
+    <t>According to Chapter 17, passing tests does not guarantee customer acceptance. Validation must also be considered.</t>
+  </si>
+  <si>
+    <t>Compared the answer with course material and lecture notes.</t>
+  </si>
+  <si>
+    <t>Classified TH5 as "Both Verification and Validation" and updated the explanation.</t>
+  </si>
+  <si>
+    <t>🗹</t>
+  </si>
+  <si>
+    <t>Các prompt đều ảnh hưởng đến quyết định trong bài SWR302</t>
+  </si>
+  <si>
+    <t>Có thay đổi phân loại MoSCoW và AC sau khi xem AI</t>
+  </si>
+  <si>
+    <t>Có giải thích trong Human Delta &amp; Reflection</t>
+  </si>
+  <si>
+    <t>Có nêu quyết định cuối cùng trong mỗi entry</t>
+  </si>
+  <si>
+    <t>Có phản biện và điều chỉnh thay vì copy AI</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Có, AI đề xuất phân loại MoSCoW và tôi đã điều chỉnh lại</t>
+  </si>
+  <si>
+    <t>Có, AI gợi ý nhiều câu hỏi và tôi chọn những câu phù hợp nhất</t>
+  </si>
+  <si>
+    <t>Có, AI giải thích từng tình huống và tôi đối chiếu lại với lý thuyết môn học</t>
+  </si>
+  <si>
+    <t>Em dựa trên định nghĩa Verification và Validation trong Chapter 17 để đưa ra quyết định</t>
+  </si>
+  <si>
+    <t>Em chọn các câu hỏi tập trung vào giá trị nghiệp vụ và mức độ cần thiết của requirement</t>
+  </si>
+  <si>
+    <t>Em ưu tiên các chức năng cốt lõi để phù hợp với thời gian 8 tuần và nhóm 3 dev</t>
   </si>
 </sst>
 </file>
@@ -472,7 +547,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -548,6 +623,16 @@
       <sz val="10"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Segoe UI Symbol"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -602,7 +687,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -654,6 +739,21 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -987,7 +1087,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -995,7 +1095,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>138</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -1003,13 +1103,16 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>139</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="C7" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="9" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -1142,7 +1245,7 @@
         <v>36</v>
       </c>
       <c r="B24" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>37</v>
@@ -1153,7 +1256,7 @@
         <v>38</v>
       </c>
       <c r="B25" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>37</v>
@@ -1164,7 +1267,7 @@
         <v>39</v>
       </c>
       <c r="B26" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>37</v>
@@ -1175,7 +1278,7 @@
         <v>40</v>
       </c>
       <c r="B27" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C27" s="9" t="s">
         <v>37</v>
@@ -1254,102 +1357,134 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="99.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="7" t="s">
-        <v>51</v>
+      <c r="A4" s="7">
+        <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>52</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>36</v>
+        <v>119</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>53</v>
+        <v>120</v>
       </c>
       <c r="E4" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="99.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="7">
+        <v>2</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F4" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="G4" s="7" t="s">
+      <c r="C5" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="99.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="7">
+        <v>3</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="H4" s="7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="99.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="99.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>66</v>
-      </c>
       <c r="C6" s="7" t="s">
-        <v>67</v>
+        <v>131</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>68</v>
+        <v>132</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>69</v>
+        <v>133</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>70</v>
+        <v>134</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>71</v>
+        <v>135</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
+        <v>136</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="91.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="7">
+        <v>4</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
+      <c r="A8" s="7">
+        <v>5</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
@@ -1552,7 +1687,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="22" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1562,7 +1697,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -1572,42 +1707,42 @@
     </row>
     <row r="3" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>81</v>
+        <v>150</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>82</v>
+        <v>151</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>83</v>
+        <v>152</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>84</v>
+        <v>153</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>85</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -1774,73 +1909,73 @@
     </row>
     <row r="30" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A31" s="10" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>91</v>
+        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>94</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>97</v>
+        <v>77</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>103</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1858,14 +1993,14 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="60" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="2" max="2" width="73" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="18" t="s">
-        <v>104</v>
+        <v>84</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1873,7 +2008,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="23" t="s">
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -1881,185 +2016,195 @@
     </row>
     <row r="4" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
-        <v>111</v>
+        <v>91</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="D6" s="13"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>155</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="D7" s="13"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
-        <v>116</v>
+        <v>95</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="D8" s="13"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>119</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="D9" s="13"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+        <v>98</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="D9" s="26" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="D10" s="13"/>
+        <v>100</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="12" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>123</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
-        <v>111</v>
+        <v>91</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>113</v>
+        <v>103</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>155</v>
       </c>
       <c r="D14" s="13"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>113</v>
+        <v>104</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>155</v>
       </c>
       <c r="D15" s="13"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
-        <v>116</v>
+        <v>95</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>113</v>
+        <v>105</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>155</v>
       </c>
       <c r="D16" s="13"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="12" t="s">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>113</v>
+        <v>106</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>155</v>
       </c>
       <c r="D17" s="13"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>113</v>
+        <v>107</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>155</v>
       </c>
       <c r="D18" s="13"/>
     </row>
     <row r="20" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
-        <v>129</v>
+        <v>108</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="15" t="s">
-        <v>130</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="15" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>132</v>
+        <v>111</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
-        <v>133</v>
+        <v>112</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="60" x14ac:dyDescent="0.2">
@@ -2067,38 +2212,56 @@
         <v>43</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>134</v>
+        <v>113</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B28" s="7"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B28" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B29" s="7"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="47.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="B30" s="7"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
+        <v>55</v>
+      </c>
+      <c r="B30" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="C30" s="28" t="s">
+        <v>164</v>
+      </c>
+      <c r="D30" s="27" t="s">
+        <v>161</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>